<commit_message>
New assembly with lightrail
created the assembly with the lightrail along with its fixtures. updated the bom with the fixtures
</commit_message>
<xml_diff>
--- a/SLSS V6/SLSS V6 BoM.xlsx
+++ b/SLSS V6/SLSS V6 BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://npluk-my.sharepoint.com/personal/matthew_mcinnes_swaney_npl_co_uk/Documents/Documents/James/SLSS/SLSS V6/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\Documents\SLSS\SLSS V6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{6EB28DA1-C942-472D-98F9-9DBE1E927EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E996334-48E6-4DBE-BA75-224295A989E1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FFC293-2762-46B5-AD05-7AA609E737AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
     <t>No</t>
   </si>
@@ -56,18 +56,6 @@
     <t>Part number</t>
   </si>
   <si>
-    <t>https://uk.rs-online.com/web/p/peltier-modules/2172395</t>
-  </si>
-  <si>
-    <t>peltier</t>
-  </si>
-  <si>
-    <t>40x40mm 77w</t>
-  </si>
-  <si>
-    <t>217-2395</t>
-  </si>
-  <si>
     <t>Assembly components</t>
   </si>
   <si>
@@ -92,97 +80,22 @@
     <t>Adafruit monochrome OLED display</t>
   </si>
   <si>
-    <t>https://uk.rs-online.com/web/p/washers/0526350?gb=a</t>
-  </si>
-  <si>
-    <t>526-350</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
-    <t>Rubber washers for screw seals</t>
-  </si>
-  <si>
-    <t>rubber washer</t>
-  </si>
-  <si>
-    <t>Temp and humidity sensor</t>
-  </si>
-  <si>
-    <t>Adafruit precision and humidity sensor</t>
-  </si>
-  <si>
-    <t>https://www.adafruit.com/product/6174</t>
-  </si>
-  <si>
-    <t>Thermocouple</t>
-  </si>
-  <si>
-    <t>Thermocouple for heatsinks</t>
-  </si>
-  <si>
-    <t>https://uk.rs-online.com/web/p/thermocouples/6212170</t>
-  </si>
-  <si>
-    <t>621-2170</t>
-  </si>
-  <si>
-    <t>https://uk.rs-online.com/web/p/uvc-lamps/2411306</t>
-  </si>
-  <si>
-    <t>241-1306</t>
-  </si>
-  <si>
-    <t>UVC Light</t>
-  </si>
-  <si>
-    <t>germocidal light</t>
-  </si>
-  <si>
-    <t>https://uk.rs-online.com/web/p/heatsinks/1846719</t>
-  </si>
-  <si>
-    <t>30mm heatsink</t>
-  </si>
-  <si>
-    <t>Heatsink</t>
-  </si>
-  <si>
-    <t>184-6719</t>
-  </si>
-  <si>
-    <t>RGB LED SMD</t>
-  </si>
-  <si>
-    <t>LED</t>
-  </si>
-  <si>
-    <t>Kingbright3.2 V, 4.1 V, 4.5 V RGB LED 5050 SMD, KAAF-5050RGBS-13 | RS</t>
-  </si>
-  <si>
-    <t>872-1724</t>
-  </si>
-  <si>
-    <t>ADV-031-11-17-E-C2 | Adaptive Peltier Module, 9 W, 3.7 A, 3.9V x 15mm | RS</t>
-  </si>
-  <si>
-    <t>606-870</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peltier </t>
-  </si>
-  <si>
-    <t xml:space="preserve">15x15mm 9w  Peltier for dehumidifier </t>
-  </si>
-  <si>
-    <t xml:space="preserve">14x14x14mm heatsink </t>
-  </si>
-  <si>
-    <t>ICK PGA 6x6x14 | Fischer Elektronik Heatsink, Universal Square Alu 14 mm 14 mm 14mm | RS</t>
-  </si>
-  <si>
-    <t>674-4740</t>
+    <t>m3x6 seal screw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSCSOR-M3-6-A2 </t>
+  </si>
+  <si>
+    <t>https://www.accu.co.uk/metric-socket-cap-head-sealing-screws/606062-SSCSOR-M3-6-A2?_gl=1*1ip1lwv*_up*MQ..*_ga*NjQzNzg0NTc2LjE3ODA3ODg3NjM.*_ga_4P9VWHTYXD*czE3ODA3ODg3NjMkbzEkZzEkdDE3ODA3ODg3NjMkajYwJGwxJGg3OTM2NjU0NDU.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHTPS-M3-5-5-S-Z </t>
+  </si>
+  <si>
+    <t>https://www.accu.co.uk/threaded-standoffs/464711-HHTPS-M3-5-5-S-Z#cad</t>
+  </si>
+  <si>
+    <t>M3Xx5x5 spacer</t>
   </si>
 </sst>
 </file>
@@ -600,15 +513,15 @@
   <dimension ref="B1:H20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="16.6328125" customWidth="1"/>
     <col min="4" max="4" width="33.54296875" customWidth="1"/>
     <col min="6" max="6" width="55.7265625" customWidth="1"/>
-    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B1" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -641,19 +554,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.35">
@@ -661,167 +571,49 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
+        <v>19</v>
+      </c>
+      <c r="E4">
+        <v>8</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>18</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5">
-        <v>6174</v>
-      </c>
+      <c r="F5" s="1"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B6">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" t="s">
-        <v>29</v>
-      </c>
+      <c r="F6" s="1"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" t="s">
-        <v>31</v>
-      </c>
+      <c r="F7" s="1"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B8">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" t="s">
-        <v>37</v>
-      </c>
+      <c r="F8" s="1"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B9">
-        <v>7</v>
-      </c>
-      <c r="C9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9">
-        <v>6</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" t="s">
-        <v>41</v>
-      </c>
+      <c r="F9" s="1"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B10">
-        <v>8</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="F10" s="1"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B11">
-        <v>9</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" t="s">
-        <v>48</v>
-      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="F11" s="1"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="F12" s="1"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" s="5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -855,16 +647,16 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.35">
@@ -872,16 +664,16 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G17" s="6">
         <v>326</v>
@@ -903,13 +695,8 @@
   <hyperlinks>
     <hyperlink ref="F16" r:id="rId1" display="https://docs.arduino.cc/resources/pinouts/ABX00028-full-pinout.pdf" xr:uid="{36804345-AEB4-4E7D-9BC7-C81B0111FE34}"/>
     <hyperlink ref="F17" r:id="rId2" location="technical-details" display="https://www.adafruit.com/product/326 - technical-details" xr:uid="{4DCB4C25-963E-47BD-BBC1-72406EC1CDC3}"/>
-    <hyperlink ref="F3" r:id="rId3" xr:uid="{A0A63F22-757F-463A-BAC4-D32816C56DA8}"/>
-    <hyperlink ref="F5" r:id="rId4" xr:uid="{354B0B53-CBFA-4FC4-B068-1AE81EC69D5D}"/>
-    <hyperlink ref="F9" r:id="rId5" display="https://uk.rs-online.com/web/p/leds/8721724" xr:uid="{368DA346-24B6-4715-9D7D-22DC54DCFC68}"/>
-    <hyperlink ref="F10" r:id="rId6" display="https://uk.rs-online.com/web/p/peltier-modules/0606870" xr:uid="{1B014EE3-9A10-47A0-948D-00A308CE41DA}"/>
-    <hyperlink ref="F11" r:id="rId7" display="https://uk.rs-online.com/web/p/heatsinks/6744740" xr:uid="{7E9861E5-040F-4EB6-850F-EFF86ACE1818}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
nut holes for watertank
</commit_message>
<xml_diff>
--- a/SLSS V6/SLSS V6 BoM.xlsx
+++ b/SLSS V6/SLSS V6 BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\Documents\SLSS\SLSS V6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://npluk-my.sharepoint.com/personal/james_edwards_npl_co_uk/Documents/Documents/SLSS/SLSS V6/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21708DCC-3D40-4B1F-8156-44C48D6B6461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{21708DCC-3D40-4B1F-8156-44C48D6B6461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA5568F4-95DB-4BB7-AD9C-DA30079A26F9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
   <si>
     <t>No</t>
   </si>
@@ -126,6 +126,30 @@
   </si>
   <si>
     <t>DC 4.5V 6V 12V 24V Tiny Mini Solenoid Valve Normally Closed N/C Flow Control Water Valve 5V Water pump</t>
+  </si>
+  <si>
+    <t>144-0700</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>Jubilee clip</t>
+  </si>
+  <si>
+    <t>1 (10)</t>
+  </si>
+  <si>
+    <t>https://uk.rs-online.com/web/p/clip-kits/1440700</t>
+  </si>
+  <si>
+    <t>336-821</t>
+  </si>
+  <si>
+    <t>Tubing</t>
   </si>
 </sst>
 </file>
@@ -578,6 +602,9 @@
       <c r="G2" t="s">
         <v>5</v>
       </c>
+      <c r="H2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3">
@@ -668,10 +695,42 @@
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="F8" s="1"/>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
       <c r="F9" s="1"/>
+      <c r="G9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C10" s="2"/>

</xml_diff>

<commit_message>
arduino and sd card placement
</commit_message>
<xml_diff>
--- a/SLSS V6/SLSS V6 BoM.xlsx
+++ b/SLSS V6/SLSS V6 BoM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://npluk-my.sharepoint.com/personal/james_edwards_npl_co_uk/Documents/Documents/SLSS/SLSS V6/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{21708DCC-3D40-4B1F-8156-44C48D6B6461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA5568F4-95DB-4BB7-AD9C-DA30079A26F9}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{21708DCC-3D40-4B1F-8156-44C48D6B6461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D50FA514-63EF-49AF-B78C-52E7252F7C6E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="63">
   <si>
     <t>No</t>
   </si>
@@ -150,6 +150,81 @@
   </si>
   <si>
     <t>Tubing</t>
+  </si>
+  <si>
+    <t>Battery holder</t>
+  </si>
+  <si>
+    <t>3x AA battery holder</t>
+  </si>
+  <si>
+    <t>RS PRO AA Battery Holder Coil Spring | RS</t>
+  </si>
+  <si>
+    <t>185-4647</t>
+  </si>
+  <si>
+    <t>883-7557</t>
+  </si>
+  <si>
+    <t>WAGO block</t>
+  </si>
+  <si>
+    <t>5 way lever connector</t>
+  </si>
+  <si>
+    <t>OLED screen</t>
+  </si>
+  <si>
+    <t>1.3 inch yellow oled screen</t>
+  </si>
+  <si>
+    <t>254-3587</t>
+  </si>
+  <si>
+    <t>MDOB128064XV-YI | Midas 1.28 in Passive matrix Yellow OLED Display 128 x 64 pixel COB I2C | RS</t>
+  </si>
+  <si>
+    <t>SD card reader</t>
+  </si>
+  <si>
+    <t>SD card reader for logging</t>
+  </si>
+  <si>
+    <t>Youmile 10 pcs SD Card Module Micro SD SDHC TF Card Adapter Reader Module with SPI Interface Level Conversion Chip with pinheader for Arduino : Amazon.co.uk: Computers &amp; Accessories</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>SSB-M2-6-A2</t>
+  </si>
+  <si>
+    <t>Accu</t>
+  </si>
+  <si>
+    <t>m2 screw</t>
+  </si>
+  <si>
+    <t>m2 screw for sd card reader</t>
+  </si>
+  <si>
+    <t>m1.4 screw</t>
+  </si>
+  <si>
+    <t>m1.4 screw for arduino nano</t>
+  </si>
+  <si>
+    <t>SIP-M1.4-10-A2</t>
+  </si>
+  <si>
+    <t>WAGO block alt</t>
+  </si>
+  <si>
+    <t>507-7011</t>
+  </si>
+  <si>
+    <t>5 way lever connector for smaller wires</t>
   </si>
 </sst>
 </file>
@@ -564,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB3D4A7C-6DC5-428F-8E7D-79698D90EF4B}">
-  <dimension ref="B1:H20"/>
+  <dimension ref="B1:H21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="16.6328125" customWidth="1"/>
@@ -622,6 +697,9 @@
       <c r="G3" t="s">
         <v>15</v>
       </c>
+      <c r="H3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4">
@@ -639,6 +717,9 @@
       <c r="G4" t="s">
         <v>17</v>
       </c>
+      <c r="H4" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5">
@@ -656,6 +737,9 @@
       <c r="G5" t="s">
         <v>25</v>
       </c>
+      <c r="H5" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B6">
@@ -673,6 +757,9 @@
       <c r="G6" t="s">
         <v>20</v>
       </c>
+      <c r="H6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7">
@@ -733,104 +820,228 @@
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="F10" s="1"/>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
+      <c r="B11">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" t="s">
+        <v>34</v>
+      </c>
       <c r="F11" s="1"/>
+      <c r="G11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="F12" s="1"/>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B13">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
+      <c r="B14">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="G14" t="s">
+        <v>53</v>
+      </c>
+      <c r="H14" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
-        <v>0</v>
+      <c r="B15">
+        <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>2</v>
-      </c>
-      <c r="E15" t="s">
-        <v>3</v>
-      </c>
-      <c r="F15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15">
         <v>4</v>
       </c>
       <c r="G15" t="s">
-        <v>5</v>
-      </c>
-      <c r="H15" s="1"/>
+        <v>59</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>62</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B18" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" t="s">
+        <v>4</v>
+      </c>
+      <c r="G19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B17">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B21">
         <v>2</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C21" t="s">
         <v>12</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D21" t="s">
         <v>13</v>
       </c>
-      <c r="E17">
+      <c r="E21">
         <v>1</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G21" s="6">
         <v>326</v>
       </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="D20" s="2"/>
-      <c r="F20" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F16" r:id="rId1" display="https://docs.arduino.cc/resources/pinouts/ABX00028-full-pinout.pdf" xr:uid="{36804345-AEB4-4E7D-9BC7-C81B0111FE34}"/>
-    <hyperlink ref="F17" r:id="rId2" location="technical-details" display="https://www.adafruit.com/product/326 - technical-details" xr:uid="{4DCB4C25-963E-47BD-BBC1-72406EC1CDC3}"/>
+    <hyperlink ref="F20" r:id="rId1" display="https://docs.arduino.cc/resources/pinouts/ABX00028-full-pinout.pdf" xr:uid="{36804345-AEB4-4E7D-9BC7-C81B0111FE34}"/>
+    <hyperlink ref="F21" r:id="rId2" location="technical-details" display="https://www.adafruit.com/product/326 - technical-details" xr:uid="{4DCB4C25-963E-47BD-BBC1-72406EC1CDC3}"/>
+    <hyperlink ref="F10" r:id="rId3" display="https://uk.rs-online.com/web/p/battery-holders/1854647" xr:uid="{9521DDEA-38F0-4C9B-93D2-026EF06185F3}"/>
+    <hyperlink ref="F12" r:id="rId4" display="https://uk.rs-online.com/web/p/oled-displays/2543587" xr:uid="{735C26EA-357D-4045-9841-B353297B07E6}"/>
+    <hyperlink ref="F13" r:id="rId5" display="https://www.amazon.co.uk/Youmile-Adapter-Interface-Conversion-pinheader/dp/B0C6KB34GZ/ref=sr_1_2_sspa?adgrpid=1175378829251379&amp;dib=eyJ2IjoiMSJ9.4G6Ta0nHdTLEh2FocR_6LAopYVw4r2qMzhRCDT8wuntULpYMdpu6Nx0Be-yz8Bj9e9U26IGfEcWXQyRzuzmArJG2SmYsuic1ec-oTgGdOdXSJYU02rsaO30kc5AMmWBO2ToZD0-HwJQ0kFMAQ_JhSWGUdU_aVZCU3bqjRWrfp9hgZlz6zhLWVtaBsl9FhPPzi88WScDckO5v8_0yqNFwJueiIPTQoT8aGONiikb1_Y4.B15R7p4uyFc5DNnBMFue4rskW8Z0N7_tFr-4B-ExBhk&amp;dib_tag=se&amp;gb=2&amp;hvadid=73461375099874&amp;hvbmt=be&amp;hvdev=c&amp;hvexpln=0&amp;hvlocphy=247141&amp;hvnetw=o&amp;hvocijid=15363587760079059900--&amp;hvqmt=e&amp;hvtargid=kwd-73461312780525%3Aloc-188&amp;hydadcr=13504_1855336&amp;keywords=arduino+micro+sd+card+module&amp;mcid=16b5a40d7175347296a474d6f7b883e3&amp;qid=1786454835&amp;sr=8-2-spons&amp;aref=HuQ1cV2wpw&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{89E43225-4AEF-4BE0-8D27-A8DAACFCBDE6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>